<commit_message>
chore(evidence): v5 scale simulation generator feeds the test assets (P8)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/evidence/2026-10-22_simulasi_skala_umkm/K1_bengkel_Bengkel_Jaya_Motor.xlsx
+++ b/docs/evidence/2026-10-22_simulasi_skala_umkm/K1_bengkel_Bengkel_Jaya_Motor.xlsx
@@ -11,8 +11,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transaksi" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rencana Anggaran" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Produk" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resep Produk" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stok Barang" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Satuan Jual" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resep Produk" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Produksi &amp; Stok" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stok Barang" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -456,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2120"/>
+  <dimension ref="A1:L2120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -503,6 +505,21 @@
       <c r="I1" t="inlineStr">
         <is>
           <t>Umur Pakai (bulan)</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Satuan</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Bahan</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Harga Satuan (Rp)</t>
         </is>
       </c>
     </row>
@@ -55497,12 +55514,12 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Satuan</t>
+          <t>Satuan Dasar</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Harga Jual (Rp)</t>
+          <t>Hasil per Batch</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -55528,7 +55545,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>95000</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
         <v>468</v>
@@ -55549,7 +55566,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>320000</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
         <v>130</v>
@@ -55570,7 +55587,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>70000</v>
+        <v>1</v>
       </c>
       <c r="D4" t="n">
         <v>572</v>
@@ -55591,7 +55608,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>20000</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
         <v>260</v>
@@ -55622,17 +55639,17 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Komponen</t>
+          <t>Satuan</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Biaya (Rp)</t>
+          <t>Isi (satuan dasar)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Untuk Berapa Unit</t>
+          <t>Harga Jual (Rp)</t>
         </is>
       </c>
     </row>
@@ -55644,14 +55661,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Oli dan bahan habis</t>
+          <t>servis</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>24000</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>95000</v>
       </c>
     </row>
     <row r="3">
@@ -55662,14 +55679,14 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Oli dan bahan habis</t>
+          <t>servis</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>80000</v>
+        <v>1</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>320000</v>
       </c>
     </row>
     <row r="4">
@@ -55680,14 +55697,14 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Oli dan bahan habis</t>
+          <t>servis</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>17500</v>
+        <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="5">
@@ -55698,14 +55715,14 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Oli dan bahan habis</t>
+          <t>servis</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>5000</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>20000</v>
       </c>
     </row>
   </sheetData>
@@ -55719,12 +55736,159 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Produk</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Komponen</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Bahan</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Jumlah per Batch</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Biaya per Batch (Rp)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Servis ringan</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Oli dan bahan habis</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>24000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Servis besar</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Oli dan bahan habis</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>80000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ganti oli</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Oli dan bahan habis</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>17500</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Tambal ban</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Oli dan bahan habis</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Tanggal</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Produk</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Jenis</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Jumlah (satuan dasar)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Catatan</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
           <t>Nama</t>
         </is>
       </c>
@@ -55746,6 +55910,11 @@
       <c r="E1" t="inlineStr">
         <is>
           <t>Batas Minimum</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Diarsipkan</t>
         </is>
       </c>
     </row>

</xml_diff>